<commit_message>
SRA sheets checked against the Hoffman FASTQ inventory; inventory script fixes
Parent panel is single-lane (L001 only), 2 files per library; pools 4.
sra_inventory.sh sorted its header into the data and split paths on
spaces; both fixed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sra/sra_metadata_all.xlsx
+++ b/sra/sra_metadata_all.xlsx
@@ -30933,16 +30933,8 @@
           <t>A1ref_Sample001_S1_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N386" t="inlineStr">
-        <is>
-          <t>A1ref_Sample001_S1_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O386" t="inlineStr">
-        <is>
-          <t>A1ref_Sample001_S1_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N386" t="inlineStr"/>
+      <c r="O386" t="inlineStr"/>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
@@ -31010,16 +31002,8 @@
           <t>A1ref_Sample002_S2_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N387" t="inlineStr">
-        <is>
-          <t>A1ref_Sample002_S2_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O387" t="inlineStr">
-        <is>
-          <t>A1ref_Sample002_S2_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N387" t="inlineStr"/>
+      <c r="O387" t="inlineStr"/>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
@@ -31087,16 +31071,8 @@
           <t>A1ref_Sample003_S3_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N388" t="inlineStr">
-        <is>
-          <t>A1ref_Sample003_S3_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O388" t="inlineStr">
-        <is>
-          <t>A1ref_Sample003_S3_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N388" t="inlineStr"/>
+      <c r="O388" t="inlineStr"/>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
@@ -31164,16 +31140,8 @@
           <t>A1ref_Sample004_S4_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N389" t="inlineStr">
-        <is>
-          <t>A1ref_Sample004_S4_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O389" t="inlineStr">
-        <is>
-          <t>A1ref_Sample004_S4_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N389" t="inlineStr"/>
+      <c r="O389" t="inlineStr"/>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
@@ -31241,16 +31209,8 @@
           <t>A1ref_Sample005_S5_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N390" t="inlineStr">
-        <is>
-          <t>A1ref_Sample005_S5_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O390" t="inlineStr">
-        <is>
-          <t>A1ref_Sample005_S5_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N390" t="inlineStr"/>
+      <c r="O390" t="inlineStr"/>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
@@ -31318,16 +31278,8 @@
           <t>A1ref_Sample006_S6_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N391" t="inlineStr">
-        <is>
-          <t>A1ref_Sample006_S6_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O391" t="inlineStr">
-        <is>
-          <t>A1ref_Sample006_S6_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N391" t="inlineStr"/>
+      <c r="O391" t="inlineStr"/>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
@@ -31395,16 +31347,8 @@
           <t>A1ref_Sample007_S7_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N392" t="inlineStr">
-        <is>
-          <t>A1ref_Sample007_S7_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O392" t="inlineStr">
-        <is>
-          <t>A1ref_Sample007_S7_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N392" t="inlineStr"/>
+      <c r="O392" t="inlineStr"/>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
@@ -31472,16 +31416,8 @@
           <t>A1ref_Sample008_S8_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N393" t="inlineStr">
-        <is>
-          <t>A1ref_Sample008_S8_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O393" t="inlineStr">
-        <is>
-          <t>A1ref_Sample008_S8_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N393" t="inlineStr"/>
+      <c r="O393" t="inlineStr"/>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
@@ -31549,16 +31485,8 @@
           <t>A1ref_Sample009_S9_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N394" t="inlineStr">
-        <is>
-          <t>A1ref_Sample009_S9_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O394" t="inlineStr">
-        <is>
-          <t>A1ref_Sample009_S9_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N394" t="inlineStr"/>
+      <c r="O394" t="inlineStr"/>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
@@ -31626,16 +31554,8 @@
           <t>A1ref_Sample013_S13_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N395" t="inlineStr">
-        <is>
-          <t>A1ref_Sample013_S13_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O395" t="inlineStr">
-        <is>
-          <t>A1ref_Sample013_S13_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N395" t="inlineStr"/>
+      <c r="O395" t="inlineStr"/>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
@@ -31703,16 +31623,8 @@
           <t>A1ref_Sample014_S14_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N396" t="inlineStr">
-        <is>
-          <t>A1ref_Sample014_S14_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O396" t="inlineStr">
-        <is>
-          <t>A1ref_Sample014_S14_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N396" t="inlineStr"/>
+      <c r="O396" t="inlineStr"/>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
@@ -31780,16 +31692,8 @@
           <t>A1ref_Sample015_S15_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N397" t="inlineStr">
-        <is>
-          <t>A1ref_Sample015_S15_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O397" t="inlineStr">
-        <is>
-          <t>A1ref_Sample015_S15_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N397" t="inlineStr"/>
+      <c r="O397" t="inlineStr"/>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
@@ -31857,16 +31761,8 @@
           <t>A1ref_Sample016_S16_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N398" t="inlineStr">
-        <is>
-          <t>A1ref_Sample016_S16_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O398" t="inlineStr">
-        <is>
-          <t>A1ref_Sample016_S16_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N398" t="inlineStr"/>
+      <c r="O398" t="inlineStr"/>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
@@ -31934,16 +31830,8 @@
           <t>A1ref_Sample017_S17_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N399" t="inlineStr">
-        <is>
-          <t>A1ref_Sample017_S17_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O399" t="inlineStr">
-        <is>
-          <t>A1ref_Sample017_S17_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N399" t="inlineStr"/>
+      <c r="O399" t="inlineStr"/>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
@@ -32011,16 +31899,8 @@
           <t>A1ref_Sample018_S18_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N400" t="inlineStr">
-        <is>
-          <t>A1ref_Sample018_S18_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O400" t="inlineStr">
-        <is>
-          <t>A1ref_Sample018_S18_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N400" t="inlineStr"/>
+      <c r="O400" t="inlineStr"/>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
@@ -32088,16 +31968,8 @@
           <t>A1ref_Sample019_S19_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N401" t="inlineStr">
-        <is>
-          <t>A1ref_Sample019_S19_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O401" t="inlineStr">
-        <is>
-          <t>A1ref_Sample019_S19_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N401" t="inlineStr"/>
+      <c r="O401" t="inlineStr"/>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
@@ -32165,16 +32037,8 @@
           <t>A1ref_Sample020_S20_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N402" t="inlineStr">
-        <is>
-          <t>A1ref_Sample020_S20_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O402" t="inlineStr">
-        <is>
-          <t>A1ref_Sample020_S20_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N402" t="inlineStr"/>
+      <c r="O402" t="inlineStr"/>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
@@ -32242,16 +32106,8 @@
           <t>A1ref_Sample021_S21_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N403" t="inlineStr">
-        <is>
-          <t>A1ref_Sample021_S21_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O403" t="inlineStr">
-        <is>
-          <t>A1ref_Sample021_S21_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N403" t="inlineStr"/>
+      <c r="O403" t="inlineStr"/>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
@@ -32319,16 +32175,8 @@
           <t>A1ref_Sample025_S25_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N404" t="inlineStr">
-        <is>
-          <t>A1ref_Sample025_S25_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O404" t="inlineStr">
-        <is>
-          <t>A1ref_Sample025_S25_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N404" t="inlineStr"/>
+      <c r="O404" t="inlineStr"/>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
@@ -32396,16 +32244,8 @@
           <t>A1ref_Sample026_S26_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N405" t="inlineStr">
-        <is>
-          <t>A1ref_Sample026_S26_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O405" t="inlineStr">
-        <is>
-          <t>A1ref_Sample026_S26_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N405" t="inlineStr"/>
+      <c r="O405" t="inlineStr"/>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
@@ -32473,16 +32313,8 @@
           <t>A1ref_Sample027_S27_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N406" t="inlineStr">
-        <is>
-          <t>A1ref_Sample027_S27_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O406" t="inlineStr">
-        <is>
-          <t>A1ref_Sample027_S27_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N406" t="inlineStr"/>
+      <c r="O406" t="inlineStr"/>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
@@ -32550,16 +32382,8 @@
           <t>A1ref_Sample028_S28_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N407" t="inlineStr">
-        <is>
-          <t>A1ref_Sample028_S28_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O407" t="inlineStr">
-        <is>
-          <t>A1ref_Sample028_S28_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N407" t="inlineStr"/>
+      <c r="O407" t="inlineStr"/>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
@@ -32627,16 +32451,8 @@
           <t>A1ref_Sample029_S29_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N408" t="inlineStr">
-        <is>
-          <t>A1ref_Sample029_S29_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O408" t="inlineStr">
-        <is>
-          <t>A1ref_Sample029_S29_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N408" t="inlineStr"/>
+      <c r="O408" t="inlineStr"/>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
@@ -32704,16 +32520,8 @@
           <t>A1ref_Sample030_S30_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N409" t="inlineStr">
-        <is>
-          <t>A1ref_Sample030_S30_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O409" t="inlineStr">
-        <is>
-          <t>A1ref_Sample030_S30_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N409" t="inlineStr"/>
+      <c r="O409" t="inlineStr"/>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
@@ -32781,16 +32589,8 @@
           <t>A1ref_Sample031_S31_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N410" t="inlineStr">
-        <is>
-          <t>A1ref_Sample031_S31_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O410" t="inlineStr">
-        <is>
-          <t>A1ref_Sample031_S31_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N410" t="inlineStr"/>
+      <c r="O410" t="inlineStr"/>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
@@ -32858,16 +32658,8 @@
           <t>A1ref_Sample032_S32_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N411" t="inlineStr">
-        <is>
-          <t>A1ref_Sample032_S32_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O411" t="inlineStr">
-        <is>
-          <t>A1ref_Sample032_S32_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N411" t="inlineStr"/>
+      <c r="O411" t="inlineStr"/>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
@@ -32935,16 +32727,8 @@
           <t>A1ref_Sample033_S33_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N412" t="inlineStr">
-        <is>
-          <t>A1ref_Sample033_S33_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O412" t="inlineStr">
-        <is>
-          <t>A1ref_Sample033_S33_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N412" t="inlineStr"/>
+      <c r="O412" t="inlineStr"/>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
@@ -33012,16 +32796,8 @@
           <t>A1ref_Sample037_S37_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N413" t="inlineStr">
-        <is>
-          <t>A1ref_Sample037_S37_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O413" t="inlineStr">
-        <is>
-          <t>A1ref_Sample037_S37_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N413" t="inlineStr"/>
+      <c r="O413" t="inlineStr"/>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
@@ -33089,16 +32865,8 @@
           <t>A1ref_Sample038_S38_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N414" t="inlineStr">
-        <is>
-          <t>A1ref_Sample038_S38_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O414" t="inlineStr">
-        <is>
-          <t>A1ref_Sample038_S38_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N414" t="inlineStr"/>
+      <c r="O414" t="inlineStr"/>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
@@ -33166,16 +32934,8 @@
           <t>A1ref_Sample039_S39_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N415" t="inlineStr">
-        <is>
-          <t>A1ref_Sample039_S39_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O415" t="inlineStr">
-        <is>
-          <t>A1ref_Sample039_S39_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N415" t="inlineStr"/>
+      <c r="O415" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
@@ -33243,16 +33003,8 @@
           <t>A1ref_Sample040_S40_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N416" t="inlineStr">
-        <is>
-          <t>A1ref_Sample040_S40_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O416" t="inlineStr">
-        <is>
-          <t>A1ref_Sample040_S40_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N416" t="inlineStr"/>
+      <c r="O416" t="inlineStr"/>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
@@ -33320,16 +33072,8 @@
           <t>A1ref_Sample041_S41_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N417" t="inlineStr">
-        <is>
-          <t>A1ref_Sample041_S41_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O417" t="inlineStr">
-        <is>
-          <t>A1ref_Sample041_S41_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N417" t="inlineStr"/>
+      <c r="O417" t="inlineStr"/>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
@@ -33397,16 +33141,8 @@
           <t>A1ref_Sample042_S42_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N418" t="inlineStr">
-        <is>
-          <t>A1ref_Sample042_S42_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O418" t="inlineStr">
-        <is>
-          <t>A1ref_Sample042_S42_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N418" t="inlineStr"/>
+      <c r="O418" t="inlineStr"/>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
@@ -33474,16 +33210,8 @@
           <t>A1ref_Sample043_S43_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N419" t="inlineStr">
-        <is>
-          <t>A1ref_Sample043_S43_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O419" t="inlineStr">
-        <is>
-          <t>A1ref_Sample043_S43_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N419" t="inlineStr"/>
+      <c r="O419" t="inlineStr"/>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
@@ -33551,16 +33279,8 @@
           <t>A1ref_Sample044_S44_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N420" t="inlineStr">
-        <is>
-          <t>A1ref_Sample044_S44_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O420" t="inlineStr">
-        <is>
-          <t>A1ref_Sample044_S44_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N420" t="inlineStr"/>
+      <c r="O420" t="inlineStr"/>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
@@ -33628,16 +33348,8 @@
           <t>A1ref_Sample045_S45_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N421" t="inlineStr">
-        <is>
-          <t>A1ref_Sample045_S45_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O421" t="inlineStr">
-        <is>
-          <t>A1ref_Sample045_S45_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N421" t="inlineStr"/>
+      <c r="O421" t="inlineStr"/>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
@@ -33705,16 +33417,8 @@
           <t>A1ref_Sample061_S61_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N422" t="inlineStr">
-        <is>
-          <t>A1ref_Sample061_S61_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O422" t="inlineStr">
-        <is>
-          <t>A1ref_Sample061_S61_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N422" t="inlineStr"/>
+      <c r="O422" t="inlineStr"/>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
@@ -33782,16 +33486,8 @@
           <t>A1ref_Sample062_S62_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N423" t="inlineStr">
-        <is>
-          <t>A1ref_Sample062_S62_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O423" t="inlineStr">
-        <is>
-          <t>A1ref_Sample062_S62_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N423" t="inlineStr"/>
+      <c r="O423" t="inlineStr"/>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
@@ -33859,16 +33555,8 @@
           <t>A1ref_Sample063_S63_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N424" t="inlineStr">
-        <is>
-          <t>A1ref_Sample063_S63_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O424" t="inlineStr">
-        <is>
-          <t>A1ref_Sample063_S63_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N424" t="inlineStr"/>
+      <c r="O424" t="inlineStr"/>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
@@ -33936,16 +33624,8 @@
           <t>A1ref_Sample064_S64_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N425" t="inlineStr">
-        <is>
-          <t>A1ref_Sample064_S64_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O425" t="inlineStr">
-        <is>
-          <t>A1ref_Sample064_S64_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N425" t="inlineStr"/>
+      <c r="O425" t="inlineStr"/>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
@@ -34013,16 +33693,8 @@
           <t>A1ref_Sample065_S65_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N426" t="inlineStr">
-        <is>
-          <t>A1ref_Sample065_S65_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O426" t="inlineStr">
-        <is>
-          <t>A1ref_Sample065_S65_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N426" t="inlineStr"/>
+      <c r="O426" t="inlineStr"/>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
@@ -34090,16 +33762,8 @@
           <t>A1ref_Sample066_S66_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N427" t="inlineStr">
-        <is>
-          <t>A1ref_Sample066_S66_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O427" t="inlineStr">
-        <is>
-          <t>A1ref_Sample066_S66_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N427" t="inlineStr"/>
+      <c r="O427" t="inlineStr"/>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
@@ -34167,16 +33831,8 @@
           <t>A1ref_Sample067_S67_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N428" t="inlineStr">
-        <is>
-          <t>A1ref_Sample067_S67_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O428" t="inlineStr">
-        <is>
-          <t>A1ref_Sample067_S67_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N428" t="inlineStr"/>
+      <c r="O428" t="inlineStr"/>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
@@ -34244,16 +33900,8 @@
           <t>A1ref_Sample068_S68_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N429" t="inlineStr">
-        <is>
-          <t>A1ref_Sample068_S68_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O429" t="inlineStr">
-        <is>
-          <t>A1ref_Sample068_S68_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N429" t="inlineStr"/>
+      <c r="O429" t="inlineStr"/>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
@@ -34321,16 +33969,8 @@
           <t>A1ref_Sample069_S69_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N430" t="inlineStr">
-        <is>
-          <t>A1ref_Sample069_S69_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O430" t="inlineStr">
-        <is>
-          <t>A1ref_Sample069_S69_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N430" t="inlineStr"/>
+      <c r="O430" t="inlineStr"/>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
@@ -34398,16 +34038,8 @@
           <t>A1ref_Sample073_S73_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N431" t="inlineStr">
-        <is>
-          <t>A1ref_Sample073_S73_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O431" t="inlineStr">
-        <is>
-          <t>A1ref_Sample073_S73_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N431" t="inlineStr"/>
+      <c r="O431" t="inlineStr"/>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
@@ -34475,16 +34107,8 @@
           <t>A1ref_Sample074_S74_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N432" t="inlineStr">
-        <is>
-          <t>A1ref_Sample074_S74_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O432" t="inlineStr">
-        <is>
-          <t>A1ref_Sample074_S74_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N432" t="inlineStr"/>
+      <c r="O432" t="inlineStr"/>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
@@ -34552,16 +34176,8 @@
           <t>A1ref_Sample075_S75_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N433" t="inlineStr">
-        <is>
-          <t>A1ref_Sample075_S75_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O433" t="inlineStr">
-        <is>
-          <t>A1ref_Sample075_S75_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N433" t="inlineStr"/>
+      <c r="O433" t="inlineStr"/>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
@@ -34629,16 +34245,8 @@
           <t>A1ref_Sample076_S76_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N434" t="inlineStr">
-        <is>
-          <t>A1ref_Sample076_S76_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O434" t="inlineStr">
-        <is>
-          <t>A1ref_Sample076_S76_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N434" t="inlineStr"/>
+      <c r="O434" t="inlineStr"/>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
@@ -34706,16 +34314,8 @@
           <t>A1ref_Sample077_S77_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N435" t="inlineStr">
-        <is>
-          <t>A1ref_Sample077_S77_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O435" t="inlineStr">
-        <is>
-          <t>A1ref_Sample077_S77_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N435" t="inlineStr"/>
+      <c r="O435" t="inlineStr"/>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
@@ -34783,16 +34383,8 @@
           <t>A1ref_Sample078_S78_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N436" t="inlineStr">
-        <is>
-          <t>A1ref_Sample078_S78_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O436" t="inlineStr">
-        <is>
-          <t>A1ref_Sample078_S78_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N436" t="inlineStr"/>
+      <c r="O436" t="inlineStr"/>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -34860,16 +34452,8 @@
           <t>A1ref_Sample079_S79_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N437" t="inlineStr">
-        <is>
-          <t>A1ref_Sample079_S79_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O437" t="inlineStr">
-        <is>
-          <t>A1ref_Sample079_S79_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N437" t="inlineStr"/>
+      <c r="O437" t="inlineStr"/>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -34937,16 +34521,8 @@
           <t>A1ref_Sample080_S80_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N438" t="inlineStr">
-        <is>
-          <t>A1ref_Sample080_S80_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O438" t="inlineStr">
-        <is>
-          <t>A1ref_Sample080_S80_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N438" t="inlineStr"/>
+      <c r="O438" t="inlineStr"/>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
@@ -35014,16 +34590,8 @@
           <t>A1ref_Sample081_S81_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N439" t="inlineStr">
-        <is>
-          <t>A1ref_Sample081_S81_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O439" t="inlineStr">
-        <is>
-          <t>A1ref_Sample081_S81_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N439" t="inlineStr"/>
+      <c r="O439" t="inlineStr"/>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
@@ -35091,16 +34659,8 @@
           <t>A1ref_Sample085_S85_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N440" t="inlineStr">
-        <is>
-          <t>A1ref_Sample085_S85_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O440" t="inlineStr">
-        <is>
-          <t>A1ref_Sample085_S85_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N440" t="inlineStr"/>
+      <c r="O440" t="inlineStr"/>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
@@ -35168,16 +34728,8 @@
           <t>A1ref_Sample086_S86_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N441" t="inlineStr">
-        <is>
-          <t>A1ref_Sample086_S86_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O441" t="inlineStr">
-        <is>
-          <t>A1ref_Sample086_S86_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N441" t="inlineStr"/>
+      <c r="O441" t="inlineStr"/>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
@@ -35245,16 +34797,8 @@
           <t>A1ref_Sample087_S87_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N442" t="inlineStr">
-        <is>
-          <t>A1ref_Sample087_S87_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O442" t="inlineStr">
-        <is>
-          <t>A1ref_Sample087_S87_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N442" t="inlineStr"/>
+      <c r="O442" t="inlineStr"/>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
@@ -35322,16 +34866,8 @@
           <t>A1ref_Sample088_S88_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N443" t="inlineStr">
-        <is>
-          <t>A1ref_Sample088_S88_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O443" t="inlineStr">
-        <is>
-          <t>A1ref_Sample088_S88_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N443" t="inlineStr"/>
+      <c r="O443" t="inlineStr"/>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
@@ -35399,16 +34935,8 @@
           <t>A1ref_Sample089_S89_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N444" t="inlineStr">
-        <is>
-          <t>A1ref_Sample089_S89_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O444" t="inlineStr">
-        <is>
-          <t>A1ref_Sample089_S89_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N444" t="inlineStr"/>
+      <c r="O444" t="inlineStr"/>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
@@ -35476,16 +35004,8 @@
           <t>A1ref_Sample090_S90_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N445" t="inlineStr">
-        <is>
-          <t>A1ref_Sample090_S90_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O445" t="inlineStr">
-        <is>
-          <t>A1ref_Sample090_S90_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N445" t="inlineStr"/>
+      <c r="O445" t="inlineStr"/>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -35553,16 +35073,8 @@
           <t>A1ref_Sample091_S91_L001_R2_001.fastq.gz</t>
         </is>
       </c>
-      <c r="N446" t="inlineStr">
-        <is>
-          <t>A1ref_Sample091_S91_L002_R1_001.fastq.gz</t>
-        </is>
-      </c>
-      <c r="O446" t="inlineStr">
-        <is>
-          <t>A1ref_Sample091_S91_L002_R2_001.fastq.gz</t>
-        </is>
-      </c>
+      <c r="N446" t="inlineStr"/>
+      <c r="O446" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="7">

</xml_diff>

<commit_message>
SRA: parent panel was sequenced on a NextSeq 2000 (read names @VH00910)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sra/sra_metadata_all.xlsx
+++ b/sra/sra_metadata_all.xlsx
@@ -30910,7 +30910,7 @@
       </c>
       <c r="I386" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J386" t="inlineStr">
@@ -30979,7 +30979,7 @@
       </c>
       <c r="I387" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J387" t="inlineStr">
@@ -31048,7 +31048,7 @@
       </c>
       <c r="I388" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J388" t="inlineStr">
@@ -31117,7 +31117,7 @@
       </c>
       <c r="I389" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J389" t="inlineStr">
@@ -31186,7 +31186,7 @@
       </c>
       <c r="I390" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J390" t="inlineStr">
@@ -31255,7 +31255,7 @@
       </c>
       <c r="I391" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J391" t="inlineStr">
@@ -31324,7 +31324,7 @@
       </c>
       <c r="I392" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J392" t="inlineStr">
@@ -31393,7 +31393,7 @@
       </c>
       <c r="I393" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J393" t="inlineStr">
@@ -31462,7 +31462,7 @@
       </c>
       <c r="I394" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J394" t="inlineStr">
@@ -31531,7 +31531,7 @@
       </c>
       <c r="I395" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J395" t="inlineStr">
@@ -31600,7 +31600,7 @@
       </c>
       <c r="I396" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J396" t="inlineStr">
@@ -31669,7 +31669,7 @@
       </c>
       <c r="I397" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J397" t="inlineStr">
@@ -31738,7 +31738,7 @@
       </c>
       <c r="I398" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J398" t="inlineStr">
@@ -31807,7 +31807,7 @@
       </c>
       <c r="I399" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J399" t="inlineStr">
@@ -31876,7 +31876,7 @@
       </c>
       <c r="I400" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J400" t="inlineStr">
@@ -31945,7 +31945,7 @@
       </c>
       <c r="I401" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J401" t="inlineStr">
@@ -32014,7 +32014,7 @@
       </c>
       <c r="I402" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J402" t="inlineStr">
@@ -32083,7 +32083,7 @@
       </c>
       <c r="I403" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J403" t="inlineStr">
@@ -32152,7 +32152,7 @@
       </c>
       <c r="I404" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J404" t="inlineStr">
@@ -32221,7 +32221,7 @@
       </c>
       <c r="I405" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J405" t="inlineStr">
@@ -32290,7 +32290,7 @@
       </c>
       <c r="I406" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J406" t="inlineStr">
@@ -32359,7 +32359,7 @@
       </c>
       <c r="I407" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J407" t="inlineStr">
@@ -32428,7 +32428,7 @@
       </c>
       <c r="I408" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J408" t="inlineStr">
@@ -32497,7 +32497,7 @@
       </c>
       <c r="I409" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J409" t="inlineStr">
@@ -32566,7 +32566,7 @@
       </c>
       <c r="I410" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J410" t="inlineStr">
@@ -32635,7 +32635,7 @@
       </c>
       <c r="I411" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J411" t="inlineStr">
@@ -32704,7 +32704,7 @@
       </c>
       <c r="I412" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J412" t="inlineStr">
@@ -32773,7 +32773,7 @@
       </c>
       <c r="I413" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J413" t="inlineStr">
@@ -32842,7 +32842,7 @@
       </c>
       <c r="I414" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J414" t="inlineStr">
@@ -32911,7 +32911,7 @@
       </c>
       <c r="I415" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J415" t="inlineStr">
@@ -32980,7 +32980,7 @@
       </c>
       <c r="I416" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J416" t="inlineStr">
@@ -33049,7 +33049,7 @@
       </c>
       <c r="I417" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J417" t="inlineStr">
@@ -33118,7 +33118,7 @@
       </c>
       <c r="I418" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J418" t="inlineStr">
@@ -33187,7 +33187,7 @@
       </c>
       <c r="I419" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J419" t="inlineStr">
@@ -33256,7 +33256,7 @@
       </c>
       <c r="I420" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J420" t="inlineStr">
@@ -33325,7 +33325,7 @@
       </c>
       <c r="I421" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J421" t="inlineStr">
@@ -33394,7 +33394,7 @@
       </c>
       <c r="I422" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J422" t="inlineStr">
@@ -33463,7 +33463,7 @@
       </c>
       <c r="I423" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J423" t="inlineStr">
@@ -33532,7 +33532,7 @@
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J424" t="inlineStr">
@@ -33601,7 +33601,7 @@
       </c>
       <c r="I425" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J425" t="inlineStr">
@@ -33670,7 +33670,7 @@
       </c>
       <c r="I426" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J426" t="inlineStr">
@@ -33739,7 +33739,7 @@
       </c>
       <c r="I427" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J427" t="inlineStr">
@@ -33808,7 +33808,7 @@
       </c>
       <c r="I428" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J428" t="inlineStr">
@@ -33877,7 +33877,7 @@
       </c>
       <c r="I429" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J429" t="inlineStr">
@@ -33946,7 +33946,7 @@
       </c>
       <c r="I430" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J430" t="inlineStr">
@@ -34015,7 +34015,7 @@
       </c>
       <c r="I431" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J431" t="inlineStr">
@@ -34084,7 +34084,7 @@
       </c>
       <c r="I432" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J432" t="inlineStr">
@@ -34153,7 +34153,7 @@
       </c>
       <c r="I433" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J433" t="inlineStr">
@@ -34222,7 +34222,7 @@
       </c>
       <c r="I434" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J434" t="inlineStr">
@@ -34291,7 +34291,7 @@
       </c>
       <c r="I435" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J435" t="inlineStr">
@@ -34360,7 +34360,7 @@
       </c>
       <c r="I436" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J436" t="inlineStr">
@@ -34429,7 +34429,7 @@
       </c>
       <c r="I437" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J437" t="inlineStr">
@@ -34498,7 +34498,7 @@
       </c>
       <c r="I438" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J438" t="inlineStr">
@@ -34567,7 +34567,7 @@
       </c>
       <c r="I439" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J439" t="inlineStr">
@@ -34636,7 +34636,7 @@
       </c>
       <c r="I440" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J440" t="inlineStr">
@@ -34705,7 +34705,7 @@
       </c>
       <c r="I441" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J441" t="inlineStr">
@@ -34774,7 +34774,7 @@
       </c>
       <c r="I442" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J442" t="inlineStr">
@@ -34843,7 +34843,7 @@
       </c>
       <c r="I443" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J443" t="inlineStr">
@@ -34912,7 +34912,7 @@
       </c>
       <c r="I444" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J444" t="inlineStr">
@@ -34981,7 +34981,7 @@
       </c>
       <c r="I445" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J445" t="inlineStr">
@@ -35050,7 +35050,7 @@
       </c>
       <c r="I446" t="inlineStr">
         <is>
-          <t>Illumina NovaSeq X</t>
+          <t>NextSeq 2000</t>
         </is>
       </c>
       <c r="J446" t="inlineStr">

</xml_diff>